<commit_message>
Update num.txt | 2026-03-11 08:05:25 JST
</commit_message>
<xml_diff>
--- a/docs/output.xlsx
+++ b/docs/output.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="174" uniqueCount="93">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="180" uniqueCount="96">
   <si>
     <t>回数</t>
   </si>
@@ -34,20 +34,45 @@
     <t>開催案内</t>
   </si>
   <si>
+    <t>第648回</t>
+  </si>
+  <si>
+    <t>2026年3月11日（令和8年3月11日）</t>
+  </si>
+  <si>
+    <t xml:space="preserve">１会長の選挙について_x000D_
+	２医薬品の新規薬価収載等について_x000D_
+	３最適使用推進ガイドラインについて（審議）_x000D_
+	４費用対効果評価の結果を踏まえた薬価の見直しについて_x000D_
+	５ＤＰＣにおける高額な新規の医薬品等への対応について_x000D_
+	６在宅自己注射について_x000D_
+	７最適使用推進ガイドラインについて（報告）_x000D_
+	８公知申請とされた適応外薬の保険適用について_x000D_
+	９先進医療会議からの報告について_x000D_
+</t>
+  </si>
+  <si>
+    <t>－</t>
+  </si>
+  <si>
+    <t xml:space="preserve">資料
+</t>
+  </si>
+  <si>
     <t>第647回</t>
   </si>
   <si>
     <t>2026年2月13日（令和8年2月13日）</t>
   </si>
   <si>
-    <t xml:space="preserve">※ 掲載準備中_x000D_
-</t>
-  </si>
-  <si>
-    <t>－</t>
-  </si>
-  <si>
-    <t xml:space="preserve">資料
+    <t xml:space="preserve">１答申について_x000D_
+	２再生医療等製品の保険適用について_x000D_
+	３ＤＰＣにおける高額な新規の医薬品等への対応について_x000D_
+	４薬価基準から削除する項目について_x000D_
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">議事録
 </t>
   </si>
   <si>
@@ -62,10 +87,6 @@
 ３個別改定項目について（その３）
 ４答申書の附帯意見案について（その２）
 ５その他
-</t>
-  </si>
-  <si>
-    <t xml:space="preserve">議事録
 </t>
   </si>
   <si>
@@ -741,7 +762,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F29"/>
+  <dimension ref="A1:F30"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:6">
@@ -1324,6 +1345,26 @@
         <v>9</v>
       </c>
     </row>
+    <row r="30" spans="1:6">
+      <c r="A30" t="s">
+        <v>93</v>
+      </c>
+      <c r="B30" t="s">
+        <v>94</v>
+      </c>
+      <c r="C30" t="s">
+        <v>95</v>
+      </c>
+      <c r="D30" t="s">
+        <v>14</v>
+      </c>
+      <c r="E30" t="s">
+        <v>10</v>
+      </c>
+      <c r="F30" t="s">
+        <v>9</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Update num.txt | 2026-04-08 08:11:30 JST
</commit_message>
<xml_diff>
--- a/docs/output.xlsx
+++ b/docs/output.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="180" uniqueCount="96">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="186" uniqueCount="99">
   <si>
     <t>回数</t>
   </si>
@@ -34,28 +34,48 @@
     <t>開催案内</t>
   </si>
   <si>
+    <t>第649回</t>
+  </si>
+  <si>
+    <t>2026年4月8日（令和8年4月8日）</t>
+  </si>
+  <si>
+    <t xml:space="preserve">１部会・小委員会に属する委員の指名等について
+２費用対効果評価専門組織からの報告について
+３医薬品の新規薬価収載等について
+４最適使用推進ガイドラインについて
+５ＤＰＣにおける高額な新規の医薬品等への対応について
+６在宅自己注射について
+７令和８年度改定を踏まえたＤＰＣ/ＰＤＰＳの現況について
+８令和８年度診療報酬改定における臨時的なＤＰＣ準備病院の募集について
+９調査実施小委員会からの報告について
+10答申書付帯意見に関する事項の検討の進め方について_x000D_
+11再生医療等製品の医療保険上の取扱いについて
+</t>
+  </si>
+  <si>
+    <t>－</t>
+  </si>
+  <si>
+    <t xml:space="preserve">資料
+</t>
+  </si>
+  <si>
     <t>第648回</t>
   </si>
   <si>
     <t>2026年3月11日（令和8年3月11日）</t>
   </si>
   <si>
-    <t xml:space="preserve">１会長の選挙について_x000D_
-	２医薬品の新規薬価収載等について_x000D_
-	３最適使用推進ガイドラインについて（審議）_x000D_
-	４費用対効果評価の結果を踏まえた薬価の見直しについて_x000D_
-	５ＤＰＣにおける高額な新規の医薬品等への対応について_x000D_
-	６在宅自己注射について_x000D_
-	７最適使用推進ガイドラインについて（報告）_x000D_
-	８公知申請とされた適応外薬の保険適用について_x000D_
-	９先進医療会議からの報告について_x000D_
-</t>
-  </si>
-  <si>
-    <t>－</t>
-  </si>
-  <si>
-    <t xml:space="preserve">資料
+    <t xml:space="preserve">１会長の選挙について
+２医薬品の新規薬価収載等について
+３最適使用推進ガイドラインについて（審議）
+４費用対効果評価の結果を踏まえた薬価の見直しについて
+５ＤＰＣにおける高額な新規の医薬品等への対応について
+６在宅自己注射について
+７最適使用推進ガイドラインについて（報告）
+８公知申請とされた適応外薬の保険適用について
+９先進医療会議からの報告について
 </t>
   </si>
   <si>
@@ -762,7 +782,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F30"/>
+  <dimension ref="A1:F31"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:6">
@@ -816,7 +836,7 @@
         <v>13</v>
       </c>
       <c r="D3" t="s">
-        <v>14</v>
+        <v>9</v>
       </c>
       <c r="E3" t="s">
         <v>10</v>
@@ -827,16 +847,16 @@
     </row>
     <row r="4" spans="1:6">
       <c r="A4" t="s">
+        <v>14</v>
+      </c>
+      <c r="B4" t="s">
         <v>15</v>
       </c>
-      <c r="B4" t="s">
+      <c r="C4" t="s">
         <v>16</v>
       </c>
-      <c r="C4" t="s">
-        <v>17</v>
-      </c>
       <c r="D4" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="E4" t="s">
         <v>10</v>
@@ -856,7 +876,7 @@
         <v>20</v>
       </c>
       <c r="D5" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="E5" t="s">
         <v>10</v>
@@ -876,7 +896,7 @@
         <v>23</v>
       </c>
       <c r="D6" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="E6" t="s">
         <v>10</v>
@@ -896,7 +916,7 @@
         <v>26</v>
       </c>
       <c r="D7" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="E7" t="s">
         <v>10</v>
@@ -916,7 +936,7 @@
         <v>29</v>
       </c>
       <c r="D8" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="E8" t="s">
         <v>10</v>
@@ -936,7 +956,7 @@
         <v>32</v>
       </c>
       <c r="D9" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="E9" t="s">
         <v>10</v>
@@ -956,7 +976,7 @@
         <v>35</v>
       </c>
       <c r="D10" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="E10" t="s">
         <v>10</v>
@@ -976,7 +996,7 @@
         <v>38</v>
       </c>
       <c r="D11" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="E11" t="s">
         <v>10</v>
@@ -996,7 +1016,7 @@
         <v>41</v>
       </c>
       <c r="D12" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="E12" t="s">
         <v>10</v>
@@ -1016,7 +1036,7 @@
         <v>44</v>
       </c>
       <c r="D13" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="E13" t="s">
         <v>10</v>
@@ -1036,7 +1056,7 @@
         <v>47</v>
       </c>
       <c r="D14" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="E14" t="s">
         <v>10</v>
@@ -1056,7 +1076,7 @@
         <v>50</v>
       </c>
       <c r="D15" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="E15" t="s">
         <v>10</v>
@@ -1076,7 +1096,7 @@
         <v>53</v>
       </c>
       <c r="D16" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="E16" t="s">
         <v>10</v>
@@ -1096,7 +1116,7 @@
         <v>56</v>
       </c>
       <c r="D17" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="E17" t="s">
         <v>10</v>
@@ -1116,7 +1136,7 @@
         <v>59</v>
       </c>
       <c r="D18" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="E18" t="s">
         <v>10</v>
@@ -1136,7 +1156,7 @@
         <v>62</v>
       </c>
       <c r="D19" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="E19" t="s">
         <v>10</v>
@@ -1156,7 +1176,7 @@
         <v>65</v>
       </c>
       <c r="D20" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="E20" t="s">
         <v>10</v>
@@ -1176,7 +1196,7 @@
         <v>68</v>
       </c>
       <c r="D21" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="E21" t="s">
         <v>10</v>
@@ -1196,7 +1216,7 @@
         <v>71</v>
       </c>
       <c r="D22" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="E22" t="s">
         <v>10</v>
@@ -1216,7 +1236,7 @@
         <v>74</v>
       </c>
       <c r="D23" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="E23" t="s">
         <v>10</v>
@@ -1236,7 +1256,7 @@
         <v>77</v>
       </c>
       <c r="D24" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="E24" t="s">
         <v>10</v>
@@ -1256,7 +1276,7 @@
         <v>80</v>
       </c>
       <c r="D25" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="E25" t="s">
         <v>10</v>
@@ -1276,7 +1296,7 @@
         <v>83</v>
       </c>
       <c r="D26" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="E26" t="s">
         <v>10</v>
@@ -1296,7 +1316,7 @@
         <v>86</v>
       </c>
       <c r="D27" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="E27" t="s">
         <v>10</v>
@@ -1316,7 +1336,7 @@
         <v>89</v>
       </c>
       <c r="D28" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="E28" t="s">
         <v>10</v>
@@ -1336,7 +1356,7 @@
         <v>92</v>
       </c>
       <c r="D29" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="E29" t="s">
         <v>10</v>
@@ -1356,12 +1376,32 @@
         <v>95</v>
       </c>
       <c r="D30" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="E30" t="s">
         <v>10</v>
       </c>
       <c r="F30" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="31" spans="1:6">
+      <c r="A31" t="s">
+        <v>96</v>
+      </c>
+      <c r="B31" t="s">
+        <v>97</v>
+      </c>
+      <c r="C31" t="s">
+        <v>98</v>
+      </c>
+      <c r="D31" t="s">
+        <v>17</v>
+      </c>
+      <c r="E31" t="s">
+        <v>10</v>
+      </c>
+      <c r="F31" t="s">
         <v>9</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Update num.txt | 2026-05-13 08:21:55 JST
</commit_message>
<xml_diff>
--- a/docs/output.xlsx
+++ b/docs/output.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="186" uniqueCount="99">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="192" uniqueCount="102">
   <si>
     <t>回数</t>
   </si>
@@ -32,6 +32,32 @@
   </si>
   <si>
     <t>開催案内</t>
+  </si>
+  <si>
+    <t>第650回</t>
+  </si>
+  <si>
+    <t>2026年5月13日（令和8年5月13日）</t>
+  </si>
+  <si>
+    <t xml:space="preserve">１部会・小委員会に属する委員の指名等について
+２費用対効果評価専門組織からの報告について
+３医療機器の保険適用について
+４医薬品の新規薬価収載等について
+５再生医療等製品の保険適用について
+６最適使用推進ガイドラインについて
+７費用対効果評価の結果を踏まえた薬価の見直しについて
+８ＤＰＣにおける高額な新規の医薬品等への対応について
+９在宅自己注射について
+10再生医療等製品の医療保険上の取扱いについて_x000D_
+</t>
+  </si>
+  <si>
+    <t>－</t>
+  </si>
+  <si>
+    <t xml:space="preserve">資料
+</t>
   </si>
   <si>
     <t>第649回</t>
@@ -49,15 +75,12 @@
 ７令和８年度改定を踏まえたＤＰＣ/ＰＤＰＳの現況について
 ８令和８年度診療報酬改定における臨時的なＤＰＣ準備病院の募集について
 ９調査実施小委員会からの報告について
-10答申書付帯意見に関する事項の検討の進め方について_x000D_
+10答申書附帯意見に関する事項の検討の進め方について_x000D_
 11再生医療等製品の医療保険上の取扱いについて
 </t>
   </si>
   <si>
-    <t>－</t>
-  </si>
-  <si>
-    <t xml:space="preserve">資料
+    <t xml:space="preserve">議事録
 </t>
   </si>
   <si>
@@ -89,10 +112,6 @@
 	２再生医療等製品の保険適用について_x000D_
 	３ＤＰＣにおける高額な新規の医薬品等への対応について_x000D_
 	４薬価基準から削除する項目について_x000D_
-</t>
-  </si>
-  <si>
-    <t xml:space="preserve">議事録
 </t>
   </si>
   <si>
@@ -782,7 +801,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F31"/>
+  <dimension ref="A1:F32"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:6">
@@ -836,7 +855,7 @@
         <v>13</v>
       </c>
       <c r="D3" t="s">
-        <v>9</v>
+        <v>14</v>
       </c>
       <c r="E3" t="s">
         <v>10</v>
@@ -847,16 +866,16 @@
     </row>
     <row r="4" spans="1:6">
       <c r="A4" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B4" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="C4" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="D4" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="E4" t="s">
         <v>10</v>
@@ -876,7 +895,7 @@
         <v>20</v>
       </c>
       <c r="D5" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="E5" t="s">
         <v>10</v>
@@ -896,7 +915,7 @@
         <v>23</v>
       </c>
       <c r="D6" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="E6" t="s">
         <v>10</v>
@@ -916,7 +935,7 @@
         <v>26</v>
       </c>
       <c r="D7" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="E7" t="s">
         <v>10</v>
@@ -936,7 +955,7 @@
         <v>29</v>
       </c>
       <c r="D8" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="E8" t="s">
         <v>10</v>
@@ -956,7 +975,7 @@
         <v>32</v>
       </c>
       <c r="D9" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="E9" t="s">
         <v>10</v>
@@ -976,7 +995,7 @@
         <v>35</v>
       </c>
       <c r="D10" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="E10" t="s">
         <v>10</v>
@@ -996,7 +1015,7 @@
         <v>38</v>
       </c>
       <c r="D11" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="E11" t="s">
         <v>10</v>
@@ -1016,7 +1035,7 @@
         <v>41</v>
       </c>
       <c r="D12" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="E12" t="s">
         <v>10</v>
@@ -1036,7 +1055,7 @@
         <v>44</v>
       </c>
       <c r="D13" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="E13" t="s">
         <v>10</v>
@@ -1056,7 +1075,7 @@
         <v>47</v>
       </c>
       <c r="D14" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="E14" t="s">
         <v>10</v>
@@ -1076,7 +1095,7 @@
         <v>50</v>
       </c>
       <c r="D15" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="E15" t="s">
         <v>10</v>
@@ -1096,7 +1115,7 @@
         <v>53</v>
       </c>
       <c r="D16" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="E16" t="s">
         <v>10</v>
@@ -1116,7 +1135,7 @@
         <v>56</v>
       </c>
       <c r="D17" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="E17" t="s">
         <v>10</v>
@@ -1136,7 +1155,7 @@
         <v>59</v>
       </c>
       <c r="D18" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="E18" t="s">
         <v>10</v>
@@ -1156,7 +1175,7 @@
         <v>62</v>
       </c>
       <c r="D19" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="E19" t="s">
         <v>10</v>
@@ -1176,7 +1195,7 @@
         <v>65</v>
       </c>
       <c r="D20" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="E20" t="s">
         <v>10</v>
@@ -1196,7 +1215,7 @@
         <v>68</v>
       </c>
       <c r="D21" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="E21" t="s">
         <v>10</v>
@@ -1216,7 +1235,7 @@
         <v>71</v>
       </c>
       <c r="D22" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="E22" t="s">
         <v>10</v>
@@ -1236,7 +1255,7 @@
         <v>74</v>
       </c>
       <c r="D23" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="E23" t="s">
         <v>10</v>
@@ -1256,7 +1275,7 @@
         <v>77</v>
       </c>
       <c r="D24" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="E24" t="s">
         <v>10</v>
@@ -1276,7 +1295,7 @@
         <v>80</v>
       </c>
       <c r="D25" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="E25" t="s">
         <v>10</v>
@@ -1296,7 +1315,7 @@
         <v>83</v>
       </c>
       <c r="D26" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="E26" t="s">
         <v>10</v>
@@ -1316,7 +1335,7 @@
         <v>86</v>
       </c>
       <c r="D27" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="E27" t="s">
         <v>10</v>
@@ -1336,7 +1355,7 @@
         <v>89</v>
       </c>
       <c r="D28" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="E28" t="s">
         <v>10</v>
@@ -1356,7 +1375,7 @@
         <v>92</v>
       </c>
       <c r="D29" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="E29" t="s">
         <v>10</v>
@@ -1376,7 +1395,7 @@
         <v>95</v>
       </c>
       <c r="D30" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="E30" t="s">
         <v>10</v>
@@ -1396,12 +1415,32 @@
         <v>98</v>
       </c>
       <c r="D31" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="E31" t="s">
         <v>10</v>
       </c>
       <c r="F31" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="32" spans="1:6">
+      <c r="A32" t="s">
+        <v>99</v>
+      </c>
+      <c r="B32" t="s">
+        <v>100</v>
+      </c>
+      <c r="C32" t="s">
+        <v>101</v>
+      </c>
+      <c r="D32" t="s">
+        <v>14</v>
+      </c>
+      <c r="E32" t="s">
+        <v>10</v>
+      </c>
+      <c r="F32" t="s">
         <v>9</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Update num.txt | 2026-06-24 08:23:18 JST
</commit_message>
<xml_diff>
--- a/docs/output.xlsx
+++ b/docs/output.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="192" uniqueCount="102">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="198" uniqueCount="105">
   <si>
     <t>回数</t>
   </si>
@@ -32,6 +32,29 @@
   </si>
   <si>
     <t>開催案内</t>
+  </si>
+  <si>
+    <t>第651回</t>
+  </si>
+  <si>
+    <t>2026年6月24日（令和8年6月24日）</t>
+  </si>
+  <si>
+    <t xml:space="preserve">１入院・外来医療等の調査・評価分科会からの報告について
+２費用対効果評価専門組織からの報告について
+３医療機器及び臨床検査の保険適用について
+４再生医療等製品の医療保険上の取扱いについて
+５最適使用推進ガイドラインについて(報告)
+６診療報酬改定結果検証部会からの報告について
+７先進医療会議からの報告について
+</t>
+  </si>
+  <si>
+    <t>－</t>
+  </si>
+  <si>
+    <t xml:space="preserve">資料
+</t>
   </si>
   <si>
     <t>第650回</t>
@@ -53,10 +76,7 @@
 </t>
   </si>
   <si>
-    <t>－</t>
-  </si>
-  <si>
-    <t xml:space="preserve">資料
+    <t xml:space="preserve">議事録
 </t>
   </si>
   <si>
@@ -77,10 +97,6 @@
 ９調査実施小委員会からの報告について
 10答申書附帯意見に関する事項の検討の進め方について_x000D_
 11再生医療等製品の医療保険上の取扱いについて
-</t>
-  </si>
-  <si>
-    <t xml:space="preserve">議事録
 </t>
   </si>
   <si>
@@ -801,7 +817,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F32"/>
+  <dimension ref="A1:F33"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:6">
@@ -1444,6 +1460,26 @@
         <v>9</v>
       </c>
     </row>
+    <row r="33" spans="1:6">
+      <c r="A33" t="s">
+        <v>102</v>
+      </c>
+      <c r="B33" t="s">
+        <v>103</v>
+      </c>
+      <c r="C33" t="s">
+        <v>104</v>
+      </c>
+      <c r="D33" t="s">
+        <v>14</v>
+      </c>
+      <c r="E33" t="s">
+        <v>10</v>
+      </c>
+      <c r="F33" t="s">
+        <v>9</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Update num.txt | 2026-07-08 08:19:08 JST
</commit_message>
<xml_diff>
--- a/docs/output.xlsx
+++ b/docs/output.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="198" uniqueCount="105">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="204" uniqueCount="108">
   <si>
     <t>回数</t>
   </si>
@@ -32,6 +32,29 @@
   </si>
   <si>
     <t>開催案内</t>
+  </si>
+  <si>
+    <t>第652回</t>
+  </si>
+  <si>
+    <t>2026年7月8日（令和8年7月8日）</t>
+  </si>
+  <si>
+    <t xml:space="preserve">１部会・小委員会に属する委員の指名等について
+２医薬品の新規薬価収載について
+３再生医療等製品の保険適用について
+４最適使用推進ガイドラインについて
+５DPCにおける高額な新規の医薬品等への対応について
+６薬価基準から削除する項目について
+７薬価専門部会からの報告について
+</t>
+  </si>
+  <si>
+    <t>－</t>
+  </si>
+  <si>
+    <t xml:space="preserve">資料
+</t>
   </si>
   <si>
     <t>第651回</t>
@@ -47,13 +70,6 @@
 ５最適使用推進ガイドラインについて(報告)
 ６診療報酬改定結果検証部会からの報告について
 ７先進医療会議からの報告について
-</t>
-  </si>
-  <si>
-    <t>－</t>
-  </si>
-  <si>
-    <t xml:space="preserve">資料
 </t>
   </si>
   <si>
@@ -817,7 +833,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F33"/>
+  <dimension ref="A1:F34"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:6">
@@ -871,7 +887,7 @@
         <v>13</v>
       </c>
       <c r="D3" t="s">
-        <v>14</v>
+        <v>9</v>
       </c>
       <c r="E3" t="s">
         <v>10</v>
@@ -882,16 +898,16 @@
     </row>
     <row r="4" spans="1:6">
       <c r="A4" t="s">
+        <v>14</v>
+      </c>
+      <c r="B4" t="s">
         <v>15</v>
       </c>
-      <c r="B4" t="s">
+      <c r="C4" t="s">
         <v>16</v>
       </c>
-      <c r="C4" t="s">
-        <v>17</v>
-      </c>
       <c r="D4" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="E4" t="s">
         <v>10</v>
@@ -911,7 +927,7 @@
         <v>20</v>
       </c>
       <c r="D5" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="E5" t="s">
         <v>10</v>
@@ -931,7 +947,7 @@
         <v>23</v>
       </c>
       <c r="D6" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="E6" t="s">
         <v>10</v>
@@ -951,7 +967,7 @@
         <v>26</v>
       </c>
       <c r="D7" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="E7" t="s">
         <v>10</v>
@@ -971,7 +987,7 @@
         <v>29</v>
       </c>
       <c r="D8" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="E8" t="s">
         <v>10</v>
@@ -991,7 +1007,7 @@
         <v>32</v>
       </c>
       <c r="D9" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="E9" t="s">
         <v>10</v>
@@ -1011,7 +1027,7 @@
         <v>35</v>
       </c>
       <c r="D10" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="E10" t="s">
         <v>10</v>
@@ -1031,7 +1047,7 @@
         <v>38</v>
       </c>
       <c r="D11" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="E11" t="s">
         <v>10</v>
@@ -1051,7 +1067,7 @@
         <v>41</v>
       </c>
       <c r="D12" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="E12" t="s">
         <v>10</v>
@@ -1071,7 +1087,7 @@
         <v>44</v>
       </c>
       <c r="D13" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="E13" t="s">
         <v>10</v>
@@ -1091,7 +1107,7 @@
         <v>47</v>
       </c>
       <c r="D14" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="E14" t="s">
         <v>10</v>
@@ -1111,7 +1127,7 @@
         <v>50</v>
       </c>
       <c r="D15" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="E15" t="s">
         <v>10</v>
@@ -1131,7 +1147,7 @@
         <v>53</v>
       </c>
       <c r="D16" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="E16" t="s">
         <v>10</v>
@@ -1151,7 +1167,7 @@
         <v>56</v>
       </c>
       <c r="D17" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="E17" t="s">
         <v>10</v>
@@ -1171,7 +1187,7 @@
         <v>59</v>
       </c>
       <c r="D18" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="E18" t="s">
         <v>10</v>
@@ -1191,7 +1207,7 @@
         <v>62</v>
       </c>
       <c r="D19" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="E19" t="s">
         <v>10</v>
@@ -1211,7 +1227,7 @@
         <v>65</v>
       </c>
       <c r="D20" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="E20" t="s">
         <v>10</v>
@@ -1231,7 +1247,7 @@
         <v>68</v>
       </c>
       <c r="D21" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="E21" t="s">
         <v>10</v>
@@ -1251,7 +1267,7 @@
         <v>71</v>
       </c>
       <c r="D22" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="E22" t="s">
         <v>10</v>
@@ -1271,7 +1287,7 @@
         <v>74</v>
       </c>
       <c r="D23" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="E23" t="s">
         <v>10</v>
@@ -1291,7 +1307,7 @@
         <v>77</v>
       </c>
       <c r="D24" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="E24" t="s">
         <v>10</v>
@@ -1311,7 +1327,7 @@
         <v>80</v>
       </c>
       <c r="D25" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="E25" t="s">
         <v>10</v>
@@ -1331,7 +1347,7 @@
         <v>83</v>
       </c>
       <c r="D26" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="E26" t="s">
         <v>10</v>
@@ -1351,7 +1367,7 @@
         <v>86</v>
       </c>
       <c r="D27" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="E27" t="s">
         <v>10</v>
@@ -1371,7 +1387,7 @@
         <v>89</v>
       </c>
       <c r="D28" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="E28" t="s">
         <v>10</v>
@@ -1391,7 +1407,7 @@
         <v>92</v>
       </c>
       <c r="D29" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="E29" t="s">
         <v>10</v>
@@ -1411,7 +1427,7 @@
         <v>95</v>
       </c>
       <c r="D30" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="E30" t="s">
         <v>10</v>
@@ -1431,7 +1447,7 @@
         <v>98</v>
       </c>
       <c r="D31" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="E31" t="s">
         <v>10</v>
@@ -1451,7 +1467,7 @@
         <v>101</v>
       </c>
       <c r="D32" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="E32" t="s">
         <v>10</v>
@@ -1471,12 +1487,32 @@
         <v>104</v>
       </c>
       <c r="D33" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="E33" t="s">
         <v>10</v>
       </c>
       <c r="F33" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="34" spans="1:6">
+      <c r="A34" t="s">
+        <v>105</v>
+      </c>
+      <c r="B34" t="s">
+        <v>106</v>
+      </c>
+      <c r="C34" t="s">
+        <v>107</v>
+      </c>
+      <c r="D34" t="s">
+        <v>17</v>
+      </c>
+      <c r="E34" t="s">
+        <v>10</v>
+      </c>
+      <c r="F34" t="s">
         <v>9</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Update num.txt | 2026-07-22 08:17:45 JST
</commit_message>
<xml_diff>
--- a/docs/output.xlsx
+++ b/docs/output.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="204" uniqueCount="108">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="210" uniqueCount="111">
   <si>
     <t>回数</t>
   </si>
@@ -32,6 +32,26 @@
   </si>
   <si>
     <t>開催案内</t>
+  </si>
+  <si>
+    <t>第653回</t>
+  </si>
+  <si>
+    <t>2026年7月22日（令和8年7月22日）</t>
+  </si>
+  <si>
+    <t xml:space="preserve">１医療機器の保険適用について
+２再生医療等製品の保険適用について
+３歯科用貴金属価格の随時改定について
+４主な施設基準の届出状況等について
+</t>
+  </si>
+  <si>
+    <t>－</t>
+  </si>
+  <si>
+    <t xml:space="preserve">資料
+</t>
   </si>
   <si>
     <t>第652回</t>
@@ -50,13 +70,6 @@
 </t>
   </si>
   <si>
-    <t>－</t>
-  </si>
-  <si>
-    <t xml:space="preserve">資料
-</t>
-  </si>
-  <si>
     <t>第651回</t>
   </si>
   <si>
@@ -70,6 +83,10 @@
 ５最適使用推進ガイドラインについて(報告)
 ６診療報酬改定結果検証部会からの報告について
 ７先進医療会議からの報告について
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">議事録
 </t>
   </si>
   <si>
@@ -89,10 +106,6 @@
 ８ＤＰＣにおける高額な新規の医薬品等への対応について
 ９在宅自己注射について
 10再生医療等製品の医療保険上の取扱いについて_x000D_
-</t>
-  </si>
-  <si>
-    <t xml:space="preserve">議事録
 </t>
   </si>
   <si>
@@ -833,7 +846,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F34"/>
+  <dimension ref="A1:F35"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:6">
@@ -1516,6 +1529,26 @@
         <v>9</v>
       </c>
     </row>
+    <row r="35" spans="1:6">
+      <c r="A35" t="s">
+        <v>108</v>
+      </c>
+      <c r="B35" t="s">
+        <v>109</v>
+      </c>
+      <c r="C35" t="s">
+        <v>110</v>
+      </c>
+      <c r="D35" t="s">
+        <v>17</v>
+      </c>
+      <c r="E35" t="s">
+        <v>10</v>
+      </c>
+      <c r="F35" t="s">
+        <v>9</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>